<commit_message>
update election excel data with robust parser
</commit_message>
<xml_diff>
--- a/data/안산시장_득표율_현황.xlsx
+++ b/data/안산시장_득표율_현황.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="득표율 현황" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="실시간 현황" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,47 +425,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>선거구명</t>
+          <t>알림</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>후보자명</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>득표수 (표)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>득표율 (%)</t>
+          <t>힌트</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>안산시</t>
+          <t>현재 선거 데이터 접수 대기 중이거나 선관위 데이터 구조가 변동되었습니다.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>확인 중...</t>
+          <t>raw_data.json 파일은 정상 수집되었습니다.</t>
         </is>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>